<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-02 Les cinq sauts sous le pin
Réécriture vocale example4 : éclat de résine, lunettes vécues, corde.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-02.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-02.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc sous le pin</t>
+          <t>parc sous le pin, pomme de pin, résine, écorce</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, Nina, papa</t>
+          <t>Victorino, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut tourner la corde pour que Nina saute cinq fois. La corde est lourde de pluie. Ils l'essuient sur le tronc. Nina saute cinq fois.</t>
+          <t>Une goutte de résine colle au tronc. Sur l'écorce, un éclat de résine brille. Victorino veut cinq sauts, maintenant. Nina arrive. Un rire commence. Nina se tait. La corde tape l'herbe. Victorino refuse de foncer. Ils tiennent la corde, à deux. Merci vécu. Un saut trop vite. L'éclat de résine tient sur l'écorce.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une pomme de pin tombe dans l'herbe. Elle fait un petit toc. Le pin sent la résine. L'écorce est rugueuse sous la main. Un peu de sève brille au soleil. Papa décroche la corde. Le coton est encore froid. Une fourmi monte sur l'écorce. Tu as entendu le toc, Victorino ? La pomme de pin. Oui. Elle est tombée toute seule. En ce moment, Victorino tient un bout. La corde sent le coton humide. Je veux tourner. Nina saute cinq fois. Cinq fois sans s'arrêter ? Oui. On compte tout haut. Nina arrive sur le gravier. Le gravier fait criss-criss. Nina a des lunettes. Nina a les cheveux tressés. Elle porte un gilet rouge. Nina, tu sautes au milieu. Tu sautes, Nina ? Oui. Papa tient l'autre bout. La corde tourne. Elle tape l'herbe, trop lourde. Ça fait un bruit mou. Un peu de terre colle au coton. Elle ne monte pas. Elle est mouillée. On peut l'essuyer. Sur le tronc. Puis on recompte.</t>
+          <t>Une goutte de résine colle au tronc. Elle fait un petit fil, chaud et collant. Ça colle, papa ! Tu la vois, sur l'écorce ? Oui, un petit fil. Le pin sent la résine, tout près. Sur l'écorce, un éclat de résine brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une pomme de pin roule dans l'herbe. Elle fait toc, sec et rond. J'ai entendu le toc. La pomme de pin ? Oui, papa. L'écorce est rugueuse, sous la main. Elle pique un peu. Papa décroche la corde de la branche. Le coton est froid, un peu lourd. Le coton sent la pluie, Victorino ? Il est mouillé. En ce moment, Victorino tient un bout. Il veut cinq sauts, tout de suite. Je veux tourner, maintenant ! Nina saute cinq fois. Cinq fois, sans s'arrêter ? Oui, papa. On compte tout haut ? Oui, tout haut. Nina arrive sur le gravier. Le gravier fait criss-criss, sous ses pas. Nina a des lunettes. Nina a les cheveux tressés. Elle porte un gilet rouge. Nina, tu sautes au milieu ? Tu sautes, Nina ? Oui. Papa tient l'autre bout. Victorino regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nina ne dit rien. Le sourire de Nina disparaît. Tu vas au milieu, maintenant ! Nina recule d'un pas. Non. Oh. Victorino tourne la corde trop vite, tout seul. La corde tape l'herbe, trop lourde. Ça fait un bruit mou. Un peu de terre colle au coton. Elle ne monte pas ! Elle est mouillée. L'éclat de résine tremble, puis tient. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Victorino ? Oui, papa. Tes mains sont collantes, Victorino ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une pomme de pin tombe dans l'herbe. Elle fait un petit toc. Le pin sent la résine. L'écorce est rugueuse sous la main. Un peu de sève brille au soleil. Papa décroche la corde. Le coton est encore froid. Une fourmi monte sur l'écorce. Tu as entendu le toc, Victorino ? La pomme de pin. Oui. Elle est tombée toute seule. En ce moment, Victorino tient un bout. La corde sent le coton humide. Je veux tourner. Nina saute cinq fois. Cinq fois sans s'arrêter ? Oui. On compte tout haut. Nina arrive sur le gravier. Le gravier fait criss-criss. Nina a des lunettes. Nina a les cheveux tressés. Elle porte un gilet rouge. Nina, tu sautes au milieu. Tu sautes, Nina ? Oui. Papa tient l'autre bout. La corde tourne. Elle tape l'herbe, trop lourde. Ça fait un bruit mou. Un peu de terre colle au coton. Elle ne monte pas. Elle est mouillée. On peut l'essuyer. Sur le tronc. Puis on recompte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte de résine colle au tronc. Elle fait un petit fil, chaud et collant. Ça colle, papa ! Tu la vois, sur l'écorce ? Oui, un petit fil. Le pin sent la résine, tout près. Sur l'écorce, un &lt;emphasis level="moderate"&gt;éclat de résine&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une pomme de pin roule dans l'herbe. Elle fait toc, sec et rond. J'ai entendu le toc. La pomme de pin ? Oui, papa. L'écorce est rugueuse, sous la main. Elle pique un peu. Papa décroche la corde de la branche. Le coton est froid, un peu lourd. Le coton sent la pluie, Victorino ? Il est mouillé. En ce moment, Victorino tient un bout. Il veut cinq sauts, tout de suite. Je veux tourner, maintenant ! Nina saute cinq fois. Cinq fois, sans s'arrêter ? Oui, papa. On compte tout haut ? Oui, tout haut. Nina arrive sur le gravier. Le gravier fait criss-criss, sous ses pas. Nina a des lunettes. Nina a les cheveux tressés. Elle porte un gilet rouge. Nina, tu sautes au milieu ? Tu sautes, Nina ? Oui. Papa tient l'autre bout. Victorino regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nina ne dit rien. Le sourire de Nina disparaît. Tu vas au milieu, maintenant ! Nina recule d'un pas. Non. Oh. Victorino tourne la corde trop vite, tout seul. La corde tape l'herbe, trop lourde. Ça fait un bruit mou. Un peu de terre colle au coton. Elle ne monte pas ! Elle est mouillée. L'éclat de résine tremble, puis tient. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Victorino ? Oui, papa. Tes mains sont collantes, Victorino ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kenzo arrive au parc avec papa. L'herbe sent la pluie. Zoé arrive aussi. Zoé a des lunettes. Zoé a les cheveux tressés. Zoé porte un gilet rouge. Kenzo regarde. Un petit rire commence. Papa parle tout de suite. Papa dit : on ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Les lunettes aident à voir. Les cheveux sont les cheveux. L'habit tient chaud. On joue. Kenzo hoche la tête. Il va vers Zoé. Ils prennent la corde. Ils sautent. Parce qu'on ne va pas rire, le jeu continue. Papa dit encore : on ne va pas rire de l'apparence. Kenzo tend la corde. Zoé saute. Les lunettes restent sur le nez. Le gilet rouge bouge. Ils sourient. [pause]</t>
+          <t>Une goutte de résine colle au tronc. Elle fait un petit fil, chaud et collant. Ça colle, papa ! Tu la vois, sur l'écorce ? Oui, un petit fil. Le pin sent la résine, tout près. Sur l'écorce, un &lt;emphasis&gt;éclat de résine&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une pomme de pin roule dans l'herbe. Elle fait toc, sec et rond. J'ai entendu le toc. La pomme de pin ? Oui, papa. L'écorce est rugueuse, sous la main. Elle pique un peu. Papa décroche la corde de la branche. Le coton est froid, un peu lourd. Le coton sent la pluie, Victorino ? Il est mouillé. En ce moment, Victorino tient un bout. Il veut cinq sauts, tout de suite. Je veux tourner, maintenant ! Nina saute cinq fois. Cinq fois, sans s'arrêter ? Oui, papa. On compte tout haut ? Oui, tout haut. Nina arrive sur le gravier. Le gravier fait criss-criss, sous ses pas. Nina a des lunettes. Nina a les cheveux tressés. Elle porte un gilet rouge. Nina, tu sautes au milieu ? Tu sautes, Nina ? Oui. Papa tient l'autre bout. Victorino regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nina ne dit rien. Le sourire de Nina disparaît. Tu vas au milieu, maintenant ! Nina recule d'un pas. Non. Oh. Victorino tourne la corde trop vite, tout seul. La corde tape l'herbe, trop lourde. Ça fait un bruit mou. Un peu de terre colle au coton. Elle ne monte pas ! Elle est mouillée. L'éclat de résine tremble, puis tient. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Victorino ? Oui, papa. Tes mains sont collantes, Victorino ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de résine</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,46 +1321,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_cinq_sauts_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une pomme de pin tombe dans l'herbe.
-narrateur|Elle fait un petit toc.
-narrateur|Le pin sent la résine.
-narrateur|L'écorce est rugueuse sous la main.
-narrateur|Un peu de sève brille au soleil.
-narrateur|Papa décroche la corde.
-narrateur|Le coton est encore froid.
-narrateur|Une fourmi monte sur l'écorce.
-papa|Tu as entendu le toc, Victorino ?
-enfant-m|La pomme de pin.
-papa|Oui.
-papa|Elle est tombée toute seule.
+          <t>narrateur|Une goutte de résine colle au tronc.
+narrateur|Elle fait un petit fil, chaud et collant.
+enfant-m|Ça colle, papa !
+papa|Tu la vois, sur l'écorce ?
+enfant-m|Oui, un petit fil.
+narrateur|Le pin sent la résine, tout près.
+narrateur|Sur l'écorce, un éclat de résine brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Une pomme de pin roule dans l'herbe.
+narrateur|Elle fait toc, sec et rond.
+enfant-m|J'ai entendu le toc.
+papa|La pomme de pin ?
+enfant-m|Oui, papa.
+maman|L'écorce est rugueuse, sous la main.
+enfant-m|Elle pique un peu.
+narrateur|Papa décroche la corde de la branche.
+narrateur|Le coton est froid, un peu lourd.
+maman|Le coton sent la pluie, Victorino ?
+enfant-m|Il est mouillé.
 narrateur|En ce moment, Victorino tient un bout.
-narrateur|La corde sent le coton humide.
-enfant-m|Je veux tourner.
+narrateur|Il veut cinq sauts, tout de suite.
+enfant-m|Je veux tourner, maintenant !
 enfant-m|Nina saute cinq fois.
-papa|Cinq fois sans s'arrêter ?
-enfant-m|Oui.
-papa|On compte tout haut.
+papa|Cinq fois, sans s'arrêter ?
+enfant-m|Oui, papa.
+maman|On compte tout haut ?
+enfant-m|Oui, tout haut.
 narrateur|Nina arrive sur le gravier.
-narrateur|Le gravier fait criss-criss.
+narrateur|Le gravier fait criss-criss, sous ses pas.
 narrateur|Nina a des lunettes.
 narrateur|Nina a les cheveux tressés.
 narrateur|Elle porte un gilet rouge.
-papa|Nina, tu sautes au milieu.
+papa|Nina, tu sautes au milieu ?
 enfant-m|Tu sautes, Nina ?
 copine|Oui.
 narrateur|Papa tient l'autre bout.
-narrateur|La corde tourne.
-narrateur|Elle tape l'herbe, trop lourde.
+narrateur|Victorino regarde les lunettes, trop longtemps.
+narrateur|Un rire commence dans sa bouche.
+narrateur|Nina ne dit rien.
+narrateur|Le sourire de Nina disparaît.
+enfant-m|Tu vas au milieu, maintenant !
+narrateur|Nina recule d'un pas.
+copine|Non.
+enfant-m|Oh.
+narrateur|Victorino tourne la corde trop vite, tout seul.
+narrateur|La corde tape l'herbe, trop lourde.
 narrateur|Ça fait un bruit mou.
 narrateur|Un peu de terre colle au coton.
-enfant-m|Elle ne monte pas.
+enfant-m|Elle ne monte pas !
 copine|Elle est mouillée.
-papa|On peut l'essuyer.
-papa|Sur le tronc.
-papa|Puis on recompte.</t>
+narrateur|L'éclat de résine tremble, puis tient.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nina, Victorino ?
+enfant-m|Oui, papa.
+maman|Tes mains sont collantes, Victorino ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1397,12 +1425,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina a des lunettes. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Zoé a des lunettes. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1412,7 +1440,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | sauter | on joue | essuyer | pas rire</t>
+          <t>jouer | on joue | ensemble | sauter | pas rire | les cinq sauts</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1427,7 +1455,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On saute ensemble. Que fait-on ?</t>
+          <t>On joue. Nina a des lunettes. Que fait-on ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1465,7 +1493,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1476,7 +1504,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1491,34 +1519,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,17 +1565,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_joue_nina_a_des_lunettes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1576,17 +1608,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino va vers Nina. Ils essuient la corde. Vous frottez le coton. Merci, Victorino. Merci, Nina. Le tronc sent la résine. Un peu de sève colle aux doigts. La corde redevient plus légère. Elle est moins lourde. On reprend ? On reprend. Nina suit la corde des yeux. On saute. Victorino tourne tout doux. La corde siffle un tout petit peu. Nina saute une fois. Un. Encore. Tu regardes la corde, Nina.</t>
+          <t>Victorino veut les cinq sauts, tout de suite. Je tourne, maintenant ! Il avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Non. Nina reste un peu plus loin. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la corde, un instant. Il écoute le toc de la pomme de pin. Tu veux les cinq sauts avec Nina ? Papa reste à la même hauteur. Tu tiens le bout ? Nina ne dit rien, d'abord. Elle pose les mains sur le coton. Je le tiens. D'accord. Merci, Victorino. Papa a vu les deux, sous le pin. La résine colle un peu, sous les doigts. Elle est chaude. Ils essuient la corde sur le tronc. Nina tient le coton, plus près. La corde redevient plus légère, cette fois. Elle monte ! Oui. Tu la vois, la corde ? Oui, papa. Au milieu, Nina ? J'y vais. Victorino tourne, sans se presser. Nina suit la corde des yeux. Nina saute une fois. Un. Deux. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste sous le pin ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino va vers Nina. Ils essuient la corde. Vous frottez le coton. Merci, Victorino. Merci, Nina. Le tronc sent la résine. Un peu de sève colle aux doigts. La corde redevient plus légère. Elle est moins lourde. On reprend ? On reprend. Nina suit la corde des yeux. On saute. Victorino tourne tout doux. La corde siffle un tout petit peu. Nina saute une fois. Un. Encore. Tu regardes la corde, Nina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut les cinq sauts, tout de suite. Je tourne, maintenant ! Il avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Non. Nina reste un peu plus loin. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt;, un instant. Il écoute le toc de la pomme de pin. Tu veux les cinq sauts avec Nina ? Papa reste à la même hauteur. Tu tiens le bout ? Nina ne dit rien, d'abord. Elle pose les mains sur le coton. Je le tiens. D'accord. Merci, Victorino. Papa a vu les deux, sous le pin. La résine colle un peu, sous les doigts. Elle est chaude. Ils essuient la corde sur le tronc. Nina tient le coton, plus près. La corde redevient plus légère, cette fois. Elle monte ! Oui. Tu la vois, la corde ? Oui, papa. Au milieu, Nina ? J'y vais. Victorino tourne, sans se presser. Nina suit la corde des yeux. Nina saute une fois. Un. Deux. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste sous le pin ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kenzo a entendu papa. On ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Kenzo et Zoé ont joué. [pause]</t>
+          <t>Victorino veut les cinq sauts, tout de suite. Je tourne, maintenant ! Il avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Non. Nina reste un peu plus loin. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la &lt;emphasis&gt;corde&lt;/emphasis&gt;, un instant. Il écoute le toc de la pomme de pin. Tu veux les cinq sauts avec Nina ? Papa reste à la même hauteur. Tu tiens le bout ? Nina ne dit rien, d'abord. Elle pose les mains sur le coton. Je le tiens. D'accord. Merci, Victorino. Papa a vu les deux, sous le pin. La résine colle un peu, sous les doigts. Elle est chaude. Ils essuient la corde sur le tronc. Nina tient le coton, plus près. La corde redevient plus légère, cette fois. Elle monte ! Oui. Tu la vois, la corde ? Oui, papa. Au milieu, Nina ? J'y vais. Victorino tourne, sans se presser. Nina suit la corde des yeux. Nina saute une fois. Un. Deux. Le ventre de Victorino se desserre. Les épaules se relèvent un peu. On reste sous le pin ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,7 +1665,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1641,10 +1673,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,30 +1699,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>corde</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1699,10 +1731,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1715,30 +1747,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_la_corde_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino va vers Nina.
-narrateur|Ils essuient la corde.
-papa|Vous frottez le coton.
+          <t>narrateur|Victorino veut les cinq sauts, tout de suite.
+enfant-m|Je tourne, maintenant !
+narrateur|Il avance trop vite vers Nina.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Nina reste un peu plus loin.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la corde, un instant.
+narrateur|Il écoute le toc de la pomme de pin.
+papa|Tu veux les cinq sauts avec Nina ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu tiens le bout ?
+narrateur|Nina ne dit rien, d'abord.
+narrateur|Elle pose les mains sur le coton.
+copine|Je le tiens.
+enfant-m|D'accord.
 papa|Merci, Victorino.
-papa|Merci, Nina.
-narrateur|Le tronc sent la résine.
-narrateur|Un peu de sève colle aux doigts.
-narrateur|La corde redevient plus légère.
-enfant-m|Elle est moins lourde.
-enfant-m|On reprend ?
-copine|On reprend.
-papa|Nina suit la corde des yeux.
-papa|On saute.
-narrateur|Victorino tourne tout doux.
-narrateur|La corde siffle un tout petit peu.
+narrateur|Papa a vu les deux, sous le pin.
+maman|La résine colle un peu, sous les doigts.
+enfant-m|Elle est chaude.
+narrateur|Ils essuient la corde sur le tronc.
+narrateur|Nina tient le coton, plus près.
+narrateur|La corde redevient plus légère, cette fois.
+enfant-m|Elle monte !
+copine|Oui.
+papa|Tu la vois, la corde ?
+enfant-m|Oui, papa.
+maman|Au milieu, Nina ?
+copine|J'y vais.
+narrateur|Victorino tourne, sans se presser.
+narrateur|Nina suit la corde des yeux.
 narrateur|Nina saute une fois.
 copine|Un.
-enfant-m|Encore.
-papa|Tu regardes la corde, Nina.</t>
+enfant-m|Deux.
+narrateur|Le ventre de Victorino se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste sous le pin ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>corde</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina saute encore. Deux. Trois. Quatre. Le gilet rouge bouge. Les tresses tapent le dos. Les lunettes restent bien. Cinq ! Cinq ! Bravo. Tu as tourné sans t'arrêter. La corde se pose dans l'herbe. On reverse les rôles ? À toi le milieu. Nina tourne à son tour. Victorino saute. Ses chaussures font toc. C'est plus facile. Oui. La corde est sèche. Un rayon passe entre les aiguilles. Il allume le gilet rouge. La fourmi est encore sur l'écorce. La pomme de pin reste dans l'herbe. On a eu nos cinq sauts. Oui. Cinq.</t>
+          <t>Nina saute, plus vite. Trois. Quatre. Le gilet rouge bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. Cinq, maintenant ! Il tourne trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nina lâche le milieu. La corde penche vers l'herbe. Ça tombe ! Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corde, un instant. Il écoute le toc de la pomme de pin. Sur l'écorce, un éclat de résine luit. Là, sur l'écorce. Tu sautes, Nina ? Nina ne dit rien. Elle reprend le milieu, sans parler. Oui. Victorino tourne, sans se presser. Nina saute. Cinq ! Cinq ! Tu as tourné sans t'arrêter ? Oui, papa. Le gilet est chaud, Nina ? Un peu. La corde se pose dans l'herbe. On reverse les rôles ? À toi le milieu. Nina tourne à son tour. Victorino saute. Ses chaussures font toc. C'est plus facile. La corde est sèche ? Oui, papa. Un rayon passe entre les aiguilles. Il allume le gilet.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina saute encore. Deux. Trois. Quatre. Le gilet rouge bouge. Les tresses tapent le dos. Les lunettes restent bien. Cinq ! Cinq ! Bravo. Tu as tourné sans t'arrêter. La corde se pose dans l'herbe. On reverse les rôles ? À toi le milieu. Nina tourne à son tour. Victorino saute. Ses chaussures font toc. C'est plus facile. Oui. La corde est sèche. Un rayon passe entre les aiguilles. Il allume le gilet rouge. La fourmi est encore sur l'écorce. La pomme de pin reste dans l'herbe. On a eu nos cinq sauts. Oui. Cinq.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina saute, plus vite. Trois. Quatre. Le gilet rouge bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. Cinq, maintenant ! Il tourne trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nina lâche le milieu. La corde penche vers l'herbe. Ça tombe ! Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corde, un instant. Il écoute le toc de la pomme de pin. Sur l'écorce, un &lt;emphasis level="moderate"&gt;éclat de résine&lt;/emphasis&gt; luit. Là, sur l'écorce. Tu sautes, Nina ? Nina ne dit rien. Elle reprend le milieu, sans parler. Oui. Victorino tourne, sans se presser. Nina saute. Cinq ! Cinq ! Tu as tourné sans t'arrêter ? Oui, papa. Le gilet est chaud, Nina ? Un peu. La corde se pose dans l'herbe. On reverse les rôles ? À toi le milieu. Nina tourne à son tour. Victorino saute. Ses chaussures font toc. C'est plus facile. La corde est sèche ? Oui, papa. Un rayon passe entre les aiguilles. Il allume le gilet.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Kenzo pose la corde. Papa verse de l'eau. Merci, dit Zoé. [pause]</t>
+          <t>Nina saute, plus vite. Trois. Quatre. Le gilet rouge bouge. Les tresses tapent le dos. Les lunettes restent sur le nez. Cinq, maintenant ! Il tourne trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nina lâche le milieu. La corde penche vers l'herbe. Ça tombe ! Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corde, un instant. Il écoute le toc de la pomme de pin. Sur l'écorce, un &lt;emphasis&gt;éclat de résine&lt;/emphasis&gt; luit. Là, sur l'écorce. Tu sautes, Nina ? Nina ne dit rien. Elle reprend le milieu, sans parler. Oui. Victorino tourne, sans se presser. Nina saute. Cinq ! Cinq ! Tu as tourné sans t'arrêter ? Oui, papa. Le gilet est chaud, Nina ? Un peu. La corde se pose dans l'herbe. On reverse les rôles ? À toi le milieu. Nina tourne à son tour. Victorino saute. Ses chaussures font toc. C'est plus facile. La corde est sèche ? Oui, papa. Un rayon passe entre les aiguilles. Il allume le gilet. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1854,28 +1916,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de résine</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1884,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1898,20 +1964,48 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina saute encore.
-copine|Deux.
-enfant-m|Trois.
-copine|Quatre.
+          <t>narrateur|Nina saute, plus vite.
+copine|Trois.
+enfant-m|Quatre.
 narrateur|Le gilet rouge bouge.
 narrateur|Les tresses tapent le dos.
-narrateur|Les lunettes restent bien.
+narrateur|Les lunettes restent sur le nez.
+enfant-m|Cinq, maintenant !
+narrateur|Il tourne trop vite, tout de suite.
+narrateur|Il regarde les lunettes, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copine|Attends.
+narrateur|Nina lâche le milieu.
+narrateur|La corde penche vers l'herbe.
+enfant-m|Ça tombe !
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Victorino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la corde, un instant.
+narrateur|Il écoute le toc de la pomme de pin.
+narrateur|Sur l'écorce, un éclat de résine luit.
+enfant-m|Là, sur l'écorce.
+enfant-m|Tu sautes, Nina ?
+narrateur|Nina ne dit rien.
+narrateur|Elle reprend le milieu, sans parler.
+copine|Oui.
+narrateur|Victorino tourne, sans se presser.
+narrateur|Nina saute.
 copine|Cinq !
 enfant-m|Cinq !
-papa|Bravo.
-papa|Tu as tourné sans t'arrêter.
+papa|Tu as tourné sans t'arrêter ?
+enfant-m|Oui, papa.
+maman|Le gilet est chaud, Nina ?
+copine|Un peu.
 narrateur|La corde se pose dans l'herbe.
 papa|On reverse les rôles ?
 copine|À toi le milieu.
@@ -1919,15 +2013,15 @@
 narrateur|Victorino saute.
 narrateur|Ses chaussures font toc.
 enfant-m|C'est plus facile.
-papa|Oui.
-papa|La corde est sèche.
-narrateur|Un rayon passe entre les aiguilles.
-narrateur|Il allume le gilet rouge.
-narrateur|La fourmi est encore sur l'écorce.
-narrateur|La pomme de pin reste dans l'herbe.
-papa|On a eu nos cinq sauts.
-enfant-m|Oui.
-enfant-m|Cinq.</t>
+papa|La corde est sèche ?
+enfant-m|Oui, papa.
+maman|Un rayon passe entre les aiguilles.
+enfant-m|Il allume le gilet.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>corde</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2048,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La corde pend à la branche. Elle n'est plus lourde. Nina a sauté cinq fois. Oui. Vous avez eu vos cinq sauts. Le pin sent encore la résine.</t>
+          <t>Ils restent sous le pin. Maman essuie un peu de terre. On a eu les cinq sauts, papa. Tu les as vus, toi ? Oui, au milieu. On est bien, ici. Victorino tapote la corde du doigt. Elle a une trace de résine. Tu la vois, la trace ? Oui, maman. La corde est restée, Victorino. Oui, avec Nina. La corde est restée. Ça sent la résine, un peu tiède. Et le pin, maman. Oui, dans l'air. La pomme de pin reste dans l'herbe. Un éclat de résine tient sur l'écorce.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La corde pend à la branche. Elle n'est plus lourde. Nina a sauté cinq fois. Oui. Vous avez eu vos cinq sauts. Le pin sent encore la résine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent sous le pin. Maman essuie un peu de terre. On a eu les cinq sauts, papa. Tu les as vus, toi ? Oui, au milieu. On est bien, ici. Victorino tapote la corde du doigt. Elle a une trace de résine. Tu la vois, la trace ? Oui, maman. La corde est restée, Victorino. Oui, avec Nina. La corde est restée. Ça sent la résine, un peu tiède. Et le pin, maman. Oui, dans l'air. La pomme de pin reste dans l'herbe. Un &lt;emphasis level="moderate"&gt;éclat de résine&lt;/emphasis&gt; tient sur l'écorce.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent sous le pin. Maman essuie un peu de terre. On a eu les cinq sauts, papa. Tu les as vus, toi ? Oui, au milieu. On est bien, ici. Victorino tapote la corde du doigt. Elle a une trace de résine. Tu la vois, la trace ? Oui, maman. La corde est restée, Victorino. Oui, avec Nina. La corde est restée. Ça sent la résine, un peu tiède. Et le pin, maman. Oui, dans l'air. La pomme de pin reste dans l'herbe. Un &lt;emphasis&gt;éclat de résine&lt;/emphasis&gt; tient sur l'écorce.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2105,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2125,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2139,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de résine</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2162,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,29 +2175,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_ecorce; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La corde pend à la branche.
-narrateur|Elle n'est plus lourde.
-enfant-m|Nina a sauté cinq fois.
-papa|Oui.
-papa|Vous avez eu vos cinq sauts.
-narrateur|Le pin sent encore la résine.</t>
+          <t>narrateur|Ils restent sous le pin.
+narrateur|Maman essuie un peu de terre.
+enfant-m|On a eu les cinq sauts, papa.
+papa|Tu les as vus, toi ?
+enfant-m|Oui, au milieu.
+maman|On est bien, ici.
+narrateur|Victorino tapote la corde du doigt.
+enfant-m|Elle a une trace de résine.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La corde est restée, Victorino.
+enfant-m|Oui, avec Nina.
+copine|La corde est restée.
+narrateur|Ça sent la résine, un peu tiède.
+enfant-m|Et le pin, maman.
+maman|Oui, dans l'air.
+narrateur|La pomme de pin reste dans l'herbe.
+narrateur|Un éclat de résine tient sur l'écorce.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pin</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2205,6 +2324,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>